<commit_message>
fix conditional formatting, psi rendering, and version in all xlsx templates
Fixed mat sheet conditional formatting ranges (E9:F50->F9:F50, M9:N50->N9:N50),
removed erroneous R9:V9 rule, replaced Symbol-font psi with cross-platform
plain text in J8 and rich text in Q8, and bumped template version to 9.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fem/files/xslope_griffiths1.xlsx
+++ b/docs/fem/files/xslope_griffiths1.xlsx
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="156">
   <si>
     <t>X</t>
   </si>
@@ -624,6 +624,37 @@
   </si>
   <si>
     <t>soil</t>
+  </si>
+  <si>
+    <t>psi</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>s(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>psi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -7922,7 +7953,7 @@
         <v>79</v>
       </c>
       <c r="D5" s="35">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -9367,8 +9398,8 @@
       <c r="I8" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="J8" s="26" t="s">
-        <v>81</v>
+      <c r="J8" s="21" t="s">
+        <v>154</v>
       </c>
       <c r="K8" s="21" t="s">
         <v>88</v>
@@ -9389,7 +9420,7 @@
         <v>82</v>
       </c>
       <c r="Q8" s="23" t="s">
-        <v>83</v>
+        <v>155</v>
       </c>
       <c r="R8" s="25" t="s">
         <v>92</v>
@@ -10130,7 +10161,7 @@
     <mergeCell ref="W7:X7"/>
     <mergeCell ref="R7:V7"/>
   </mergeCells>
-  <conditionalFormatting sqref="E9:F50">
+  <conditionalFormatting sqref="F9:F50">
     <cfRule type="expression" dxfId="8" priority="1">
       <formula>$D9="cp"</formula>
     </cfRule>
@@ -10145,7 +10176,7 @@
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M9:N50">
+  <conditionalFormatting sqref="N9:N50">
     <cfRule type="expression" dxfId="5" priority="7">
       <formula>$D9="cp"</formula>
     </cfRule>

</xml_diff>